<commit_message>
Report v2: new DTR template with Section F cash brought forward, G cash received, H reconciliation; Cash tab and Month/Report screens updated (v0.6.0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQBQWNtRFM4orp2c2sV98o
</commit_message>
<xml_diff>
--- a/assets/templates/DTR-PUR-UTAS-NIZWA-template.xlsx
+++ b/assets/templates/DTR-PUR-UTAS-NIZWA-template.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47FC555-5636-4BB6-A526-AD60D135FF0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Purchase Report" state="visible" r:id="rId4"/>
+    <sheet name="Purchase Report" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="41">
   <si>
     <t>DARYAS TRADING AND CONTRACTING  LLC</t>
   </si>
@@ -106,92 +110,118 @@
     <t>No fuel bills recorded during the period.</t>
   </si>
   <si>
-    <t>Section F — Cash Received from Cashier</t>
-  </si>
-  <si>
     <t>Amount</t>
   </si>
   <si>
     <t>No cash received recorded during the period.</t>
   </si>
   <si>
-    <t>Section G — Reconciliation Summary</t>
-  </si>
-  <si>
     <t>TOTAL PURCHASE VALUE</t>
   </si>
   <si>
     <t>OMR</t>
   </si>
   <si>
-    <t>TOTAL CASH RECEIVED</t>
-  </si>
-  <si>
     <t>BALANCE DUE (Payable by Cashier)</t>
+  </si>
+  <si>
+    <t>Section F — Cash Brought Forward from Last Month</t>
+  </si>
+  <si>
+    <t>CASH BROUGHT FORWARD FROM LAST MONTH</t>
+  </si>
+  <si>
+    <t>CASH RECEIVED FROM CASHIER</t>
+  </si>
+  <si>
+    <t>Section G — Cash Received from Cashier</t>
+  </si>
+  <si>
+    <t>Section H— Reconciliation Summary</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF1B2430"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10.5"/>
+      <color rgb="FF1B2430"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="14"/>
       <color rgb="FF1B2430"/>
-      <sz val="16"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF1B2430"/>
-      <sz val="10.5"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF1B2430"/>
-      <sz val="14"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11.5"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11.5"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="9.5"/>
       <color rgb="FF16283F"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF5B6472"/>
-      <sz val="9.5"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <i/>
       <sz val="9.5"/>
+      <color rgb="FF5B6472"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9.5"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.5"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9.5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -244,8 +274,46 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -255,34 +323,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -621,496 +661,559 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <dimension ref="A1:I41"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="12.453125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-    </row>
-    <row r="2" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+    </row>
+    <row r="2" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="4" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+    </row>
+    <row r="4" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-    </row>
-    <row r="5" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+    </row>
+    <row r="5" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="F7" s="4" t="s">
+      <c r="C7" s="16"/>
+      <c r="F7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="F8" s="4" t="s">
+      <c r="C8" s="16"/>
+      <c r="F8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+    </row>
+    <row r="10" spans="1:9" ht="13.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+    </row>
+    <row r="14" spans="1:9" ht="13.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+    </row>
+    <row r="18" spans="1:9" ht="13.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="G19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="H19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="I19" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+    </row>
+    <row r="22" spans="1:9" ht="13.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H23" s="7" t="s">
+      <c r="H23" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I23" s="7" t="s">
+      <c r="I23" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+    </row>
+    <row r="26" spans="1:9" ht="13.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G27" s="7" t="s">
+      <c r="G27" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H27" s="7" t="s">
+      <c r="H27" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I27" s="7" t="s">
+      <c r="I27" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="8" t="s">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29" s="8"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+    </row>
+    <row r="30" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+      <c r="A30" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="9" t="s">
+      <c r="I31" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="13.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B34" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C34" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9" t="s">
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="I31" s="9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="s">
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+    </row>
+    <row r="37" spans="1:9" ht="13.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="11"/>
+      <c r="C37" s="11"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A38" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
-    </row>
-    <row r="34" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="4">
+        <v>0</v>
+      </c>
+      <c r="I38" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B39" s="12"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="4">
+        <v>0</v>
+      </c>
+      <c r="I39" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B40" s="12"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="12"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="4">
+        <v>0</v>
+      </c>
+      <c r="I40" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A41" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="11">
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="6">
         <v>0</v>
       </c>
-      <c r="I35" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="11">
-        <v>0</v>
-      </c>
-      <c r="I36" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="14">
-        <v>0</v>
-      </c>
-      <c r="I38" s="15" t="s">
-        <v>36</v>
+      <c r="I41" s="7" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="28">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A4:I4"/>
@@ -1129,15 +1232,18 @@
     <mergeCell ref="A24:I24"/>
     <mergeCell ref="A26:I26"/>
     <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A33:I33"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="A30:I30"/>
     <mergeCell ref="C31:G31"/>
-    <mergeCell ref="A32:I32"/>
-    <mergeCell ref="A34:I34"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A40:G40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>